<commit_message>
EWA - adjustment format import question
</commit_message>
<xml_diff>
--- a/public/import/Template soal CBT.xlsx
+++ b/public/import/Template soal CBT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericwahyu/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA2E226-420B-1B42-B52B-8F85A5DA7E3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{533208E8-B83B-AB4A-AAEA-D1D96311B6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1260" windowWidth="34200" windowHeight="20980" xr2:uid="{D4F72752-1A0A-F54B-8535-D42379D12992}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>Topik Soal</t>
   </si>
@@ -114,13 +114,28 @@
   </si>
   <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>Prodi</t>
+  </si>
+  <si>
+    <t>Kedokteran</t>
+  </si>
+  <si>
+    <t>PEMBERITAHUAN
+1. Pastikan Kolom Prodi, Topik Soal, Kategori Materi, dan Materi soal ada di dalam data master pada sistem, jika tidak maka data tersebut akan kosong.
+2. Kolom Tipe Soal harus sesuai dengan tipe yang ada di master data, jika tidak sama maka data soal tidak akan masuk dalam import.
+3. Kolom Soal bersifat wajib diisi.
+4. Kolom Deskripsi berisifat opsional untuk di isi.
+5. Kolom A-E adalah pilihan jawaban untuk soal tersebut dan bersifat wajib diisi.
+6. Kolom Jawaban adalah kunci jawaban dari soal tersebut.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -141,13 +156,24 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6FF49"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -177,18 +203,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF6FF49"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -517,121 +555,317 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EA10F97-AAAA-964A-A54A-D638B4672F16}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>12</v>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>27</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="P2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>20</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>22</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>23</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>24</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>25</v>
       </c>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="4"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="4"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="4"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+      <c r="U13" s="4"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
+      <c r="S14" s="4"/>
+      <c r="T14" s="4"/>
+      <c r="U14" s="4"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
+      <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="U15" s="4"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+      <c r="S16" s="4"/>
+      <c r="T16" s="4"/>
+      <c r="U16" s="4"/>
+    </row>
+    <row r="17" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P17" s="4"/>
+      <c r="Q17" s="4"/>
+      <c r="R17" s="4"/>
+      <c r="S17" s="4"/>
+      <c r="T17" s="4"/>
+      <c r="U17" s="4"/>
+    </row>
+    <row r="18" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4"/>
+      <c r="S18" s="4"/>
+      <c r="T18" s="4"/>
+      <c r="U18" s="4"/>
+    </row>
+    <row r="19" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4"/>
+      <c r="T19" s="4"/>
+      <c r="U19" s="4"/>
+    </row>
+    <row r="20" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
+      <c r="U20" s="4"/>
+    </row>
+    <row r="21" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+      <c r="S21" s="4"/>
+      <c r="T21" s="4"/>
+      <c r="U21" s="4"/>
+    </row>
+    <row r="22" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
+      <c r="S22" s="4"/>
+      <c r="T22" s="4"/>
+      <c r="U22" s="4"/>
+    </row>
+    <row r="23" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
+      <c r="R23" s="4"/>
+      <c r="S23" s="4"/>
+      <c r="T23" s="4"/>
+      <c r="U23" s="4"/>
+    </row>
+    <row r="24" spans="16:21" x14ac:dyDescent="0.2">
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
+      <c r="U24" s="4"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="P2:U24"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>